<commit_message>
rename modality to enumeration
</commit_message>
<xml_diff>
--- a/public/data/db-source/value.xlsx
+++ b/public/data/db-source/value.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFE631FD-CE0F-8D42-B8C2-F9E8817BED37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{985B490D-423E-7D48-BA95-BA1B9C455F2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,18 +22,12 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="86">
   <si>
-    <t>modality_id</t>
-  </si>
-  <si>
     <t>value</t>
   </si>
   <si>
     <t>description</t>
   </si>
   <si>
-    <t>modality_1</t>
-  </si>
-  <si>
     <t>value_1</t>
   </si>
   <si>
@@ -277,17 +271,29 @@
     <t>xyz33</t>
   </si>
   <si>
-    <t>Schwytz et autres régions d'ici et d'ailleur et de partout et de part le monde mais aussi d'ici</t>
+    <t>enumeration_id</t>
+  </si>
+  <si>
+    <t>enumeration_1</t>
+  </si>
+  <si>
+    <t>Schwytz et autres régions d'ici et d'ailleur et de partout et de part le monde mais aussi d'ici aussi</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -355,7 +361,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B6673E3E-F092-B843-96DC-BE1B5C5F51B8}" name="Tableau3" displayName="Tableau3" ref="A1:C44" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
   <autoFilter ref="A1:C44" xr:uid="{B6673E3E-F092-B843-96DC-BE1B5C5F51B8}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{F479AE5F-1828-5E4C-A23B-6285A48F29B3}" name="modality_id" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{F479AE5F-1828-5E4C-A23B-6285A48F29B3}" name="enumeration_id" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{84C4D4A2-8ACD-B045-91A5-EBA02C626C87}" name="value" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{01460B31-0589-8747-9802-8BCA0B387BD1}" name="description" dataDxfId="0"/>
   </tableColumns>
@@ -653,7 +659,7 @@
   <dimension ref="A1:C44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="16384" width="8.83203125" style="1"/>
@@ -661,103 +667,103 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>84</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>84</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B10" s="1">
         <v>0</v>
@@ -765,54 +771,54 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C15" t="s">
         <v>85</v>
@@ -820,321 +826,322 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C16" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C17" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C18" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C19" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C20" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C21" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C22" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C23" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C24" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C25" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C26" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C27" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C28" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C29" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C30" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C31" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C32" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C33" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C34" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C35" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C36" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B41" s="1">
         <v>0</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B42" s="1">
         <v>1</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
Align app terminology, add folder.link, and fix multi-line numPercent cells (#126)
* fix: multi-line `numPercent` cells (e.g. dates) collapsing to a single line after the clickable-cell change

* add folder link support

* Rename institution entity to organization

* change header navigation labels

* rename freq to frequency

* update evolution for frequency rename

* rename dataset structure sections

* rename modality to enumeration

* update version to 0.21.0
</commit_message>
<xml_diff>
--- a/public/data/db-source/value.xlsx
+++ b/public/data/db-source/value.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFE631FD-CE0F-8D42-B8C2-F9E8817BED37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{985B490D-423E-7D48-BA95-BA1B9C455F2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,18 +22,12 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="86">
   <si>
-    <t>modality_id</t>
-  </si>
-  <si>
     <t>value</t>
   </si>
   <si>
     <t>description</t>
   </si>
   <si>
-    <t>modality_1</t>
-  </si>
-  <si>
     <t>value_1</t>
   </si>
   <si>
@@ -277,17 +271,29 @@
     <t>xyz33</t>
   </si>
   <si>
-    <t>Schwytz et autres régions d'ici et d'ailleur et de partout et de part le monde mais aussi d'ici</t>
+    <t>enumeration_id</t>
+  </si>
+  <si>
+    <t>enumeration_1</t>
+  </si>
+  <si>
+    <t>Schwytz et autres régions d'ici et d'ailleur et de partout et de part le monde mais aussi d'ici aussi</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -355,7 +361,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B6673E3E-F092-B843-96DC-BE1B5C5F51B8}" name="Tableau3" displayName="Tableau3" ref="A1:C44" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
   <autoFilter ref="A1:C44" xr:uid="{B6673E3E-F092-B843-96DC-BE1B5C5F51B8}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{F479AE5F-1828-5E4C-A23B-6285A48F29B3}" name="modality_id" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{F479AE5F-1828-5E4C-A23B-6285A48F29B3}" name="enumeration_id" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{84C4D4A2-8ACD-B045-91A5-EBA02C626C87}" name="value" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{01460B31-0589-8747-9802-8BCA0B387BD1}" name="description" dataDxfId="0"/>
   </tableColumns>
@@ -653,7 +659,7 @@
   <dimension ref="A1:C44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="16384" width="8.83203125" style="1"/>
@@ -661,103 +667,103 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>84</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>84</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B10" s="1">
         <v>0</v>
@@ -765,54 +771,54 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C15" t="s">
         <v>85</v>
@@ -820,321 +826,322 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C16" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C17" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C18" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C19" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C20" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C21" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C22" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C23" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C24" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C25" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C26" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C27" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C28" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C29" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C30" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C31" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C32" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C33" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C34" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C35" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C36" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B41" s="1">
         <v>0</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B42" s="1">
         <v>1</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>